<commit_message>
Fix data-quality bugs, correct findings, and reorganize project
- Convert prose cells saved as code cells to Markdown
- Use a relative path for the raw data file (reproducible on any machine)
- Show the duplicates that were actually removed; build cleaning log from results
- Flag implausible values in a new Implausible_Flag column
- Correct overstated takeaways and report numbers to match the data
- Save charts in charts/; add requirements.txt and project brief
- Rewrite README with setup instructions and key findings

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/laboratory_patient_data_cleaned.xlsx
+++ b/laboratory_patient_data_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M501"/>
+  <dimension ref="A1:N501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,11 @@
           <t>Diabetes</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Implausible_Flag</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -527,6 +532,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -574,6 +580,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -621,6 +628,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -668,6 +676,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -715,6 +724,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -762,6 +772,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -809,6 +820,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -856,6 +868,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -903,6 +916,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -948,6 +962,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -995,6 +1010,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1042,6 +1058,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1089,6 +1106,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1136,6 +1154,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1183,6 +1202,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1230,6 +1250,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1277,6 +1298,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1324,6 +1346,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1371,6 +1394,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1418,6 +1442,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1465,6 +1490,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1512,6 +1538,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1559,6 +1586,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1606,6 +1634,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1653,6 +1682,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1700,6 +1730,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1747,6 +1778,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1794,6 +1826,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1841,6 +1874,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1888,6 +1922,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1935,6 +1970,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1982,6 +2018,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2027,6 +2064,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2074,6 +2112,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2121,6 +2160,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2168,6 +2208,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2215,6 +2256,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2262,6 +2304,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2309,6 +2352,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2356,6 +2400,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2401,6 +2446,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2448,6 +2494,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2495,6 +2542,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2540,6 +2588,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2587,6 +2636,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2634,6 +2684,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2681,6 +2732,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2726,6 +2778,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2773,6 +2826,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2820,6 +2874,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2867,6 +2922,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2914,6 +2970,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2961,6 +3018,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3008,6 +3066,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3055,6 +3114,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3102,6 +3162,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3149,6 +3210,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3196,6 +3258,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3243,6 +3306,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3290,6 +3354,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3337,6 +3402,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3384,6 +3450,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3431,6 +3498,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3478,6 +3546,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3525,6 +3594,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3572,6 +3642,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3619,6 +3690,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3666,6 +3738,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3713,6 +3786,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3760,6 +3834,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3807,6 +3882,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3854,6 +3930,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3901,6 +3978,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3948,6 +4026,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3995,6 +4074,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4042,6 +4122,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4089,6 +4170,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4136,6 +4218,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4183,6 +4266,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4230,6 +4314,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4277,6 +4362,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4324,6 +4410,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4371,6 +4458,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4416,6 +4504,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4463,6 +4552,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4510,6 +4600,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4557,6 +4648,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4604,6 +4696,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4651,6 +4744,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4698,6 +4792,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4745,6 +4840,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4792,6 +4888,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4835,6 +4932,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4880,6 +4978,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4927,6 +5026,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4974,6 +5074,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5021,6 +5122,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5068,6 +5170,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5115,6 +5218,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5162,6 +5266,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5209,6 +5314,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5256,6 +5362,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5303,6 +5410,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5348,6 +5456,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5395,6 +5504,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5442,6 +5552,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5489,6 +5600,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5536,6 +5648,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5583,6 +5696,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5630,6 +5744,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5677,6 +5792,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5722,6 +5838,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5769,6 +5886,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5816,6 +5934,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5863,6 +5982,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5910,6 +6030,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5957,6 +6078,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>Total_Cholesterol_mg_dL</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6004,6 +6130,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6051,6 +6178,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6098,6 +6226,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6145,6 +6274,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6192,6 +6322,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6239,6 +6370,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6286,6 +6418,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -6333,6 +6466,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6380,6 +6514,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -6425,6 +6560,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -6472,6 +6608,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6519,6 +6656,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6566,6 +6704,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6613,6 +6752,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6660,6 +6800,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -6705,6 +6846,11 @@
       <c r="M134" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>Age</t>
         </is>
       </c>
     </row>
@@ -6752,6 +6898,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -6799,6 +6946,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6846,6 +6994,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6893,6 +7042,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6940,6 +7090,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6987,6 +7138,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -7034,6 +7186,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -7081,6 +7234,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7128,6 +7282,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -7175,6 +7330,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -7222,6 +7378,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -7269,6 +7426,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -7316,6 +7474,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -7363,6 +7522,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -7410,6 +7570,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -7457,6 +7618,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -7504,6 +7666,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -7551,6 +7714,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -7596,6 +7760,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -7643,6 +7808,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -7690,6 +7856,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -7737,6 +7904,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -7784,6 +7952,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -7831,6 +8000,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -7878,6 +8048,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -7925,6 +8096,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -7972,6 +8144,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -8019,6 +8192,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>Total_Cholesterol_mg_dL</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -8066,6 +8244,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -8113,6 +8292,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -8160,6 +8340,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -8207,6 +8388,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -8254,6 +8436,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -8299,6 +8482,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -8346,6 +8530,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -8393,6 +8578,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -8440,6 +8626,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -8487,6 +8674,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -8534,6 +8722,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -8581,6 +8770,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -8628,6 +8818,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -8675,6 +8866,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -8722,6 +8914,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -8769,6 +8962,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -8816,6 +9010,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -8863,6 +9058,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -8908,6 +9104,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -8953,6 +9150,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -9000,6 +9198,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -9047,6 +9246,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -9094,6 +9294,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -9141,6 +9342,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -9188,6 +9390,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -9235,6 +9438,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -9282,6 +9486,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -9327,6 +9532,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -9374,6 +9580,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -9421,6 +9628,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -9468,6 +9676,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -9515,6 +9724,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -9560,6 +9770,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -9607,6 +9818,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -9654,6 +9866,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -9701,6 +9914,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -9748,6 +9962,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -9795,6 +10010,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -9842,6 +10058,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -9889,6 +10106,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -9934,6 +10152,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -9981,6 +10200,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -10028,6 +10248,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -10075,6 +10296,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -10122,6 +10344,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -10169,6 +10392,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -10216,6 +10440,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -10263,6 +10488,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -10308,6 +10534,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -10355,6 +10582,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -10402,6 +10630,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -10449,6 +10678,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -10496,6 +10726,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -10543,6 +10774,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -10590,6 +10822,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -10637,6 +10870,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -10684,6 +10918,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -10731,6 +10966,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -10778,6 +11014,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -10825,6 +11062,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -10872,6 +11110,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -10917,6 +11156,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -10964,6 +11204,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -11011,6 +11252,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -11056,6 +11298,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -11103,6 +11346,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -11148,6 +11392,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -11195,6 +11440,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -11242,6 +11488,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -11289,6 +11536,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -11336,6 +11584,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -11383,6 +11632,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -11430,6 +11680,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -11477,6 +11728,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -11524,6 +11776,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -11571,6 +11824,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -11618,6 +11872,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -11665,6 +11920,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -11712,6 +11968,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -11759,6 +12016,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -11804,6 +12062,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -11851,6 +12110,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -11898,6 +12158,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -11945,6 +12206,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -11992,6 +12254,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -12039,6 +12302,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -12086,6 +12350,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -12133,6 +12398,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -12180,6 +12446,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -12227,6 +12494,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -12274,6 +12542,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -12321,6 +12590,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -12368,6 +12638,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -12415,6 +12686,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -12462,6 +12734,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -12509,6 +12782,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -12556,6 +12830,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -12603,6 +12878,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -12650,6 +12926,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -12697,6 +12974,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -12744,6 +13022,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -12791,6 +13070,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -12838,6 +13118,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -12885,6 +13166,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -12932,6 +13214,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -12979,6 +13262,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -13026,6 +13310,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -13073,6 +13358,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -13120,6 +13406,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -13167,6 +13454,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -13214,6 +13502,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -13261,6 +13550,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -13308,6 +13598,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -13355,6 +13646,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -13402,6 +13694,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -13449,6 +13742,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -13496,6 +13790,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -13543,6 +13838,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N280" t="inlineStr">
+        <is>
+          <t>HDL_mg_dL</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -13590,6 +13890,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -13637,6 +13938,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -13684,6 +13986,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -13729,6 +14032,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -13776,6 +14080,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -13823,6 +14128,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -13868,6 +14174,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -13915,6 +14222,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -13962,6 +14270,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -14009,6 +14318,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -14056,6 +14366,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -14103,6 +14414,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -14150,6 +14462,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -14197,6 +14510,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -14244,6 +14558,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -14291,6 +14606,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -14338,6 +14654,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -14383,6 +14700,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -14430,6 +14748,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -14477,6 +14796,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -14522,6 +14842,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -14569,6 +14890,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -14616,6 +14938,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -14663,6 +14986,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -14710,6 +15034,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -14757,6 +15082,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -14804,6 +15130,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -14851,6 +15178,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -14898,6 +15226,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -14945,6 +15274,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -14990,6 +15320,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -15037,6 +15368,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -15084,6 +15416,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -15131,6 +15464,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -15176,6 +15510,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -15223,6 +15558,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -15270,6 +15606,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -15317,6 +15654,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -15364,6 +15702,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -15409,6 +15748,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -15456,6 +15796,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -15503,6 +15844,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -15550,6 +15892,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -15597,6 +15940,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -15644,6 +15988,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -15691,6 +16036,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -15736,6 +16082,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -15781,6 +16128,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -15828,6 +16176,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -15875,6 +16224,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -15922,6 +16272,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -15969,6 +16320,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -16016,6 +16368,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -16063,6 +16416,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -16110,6 +16464,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -16157,6 +16512,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -16202,6 +16558,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -16249,6 +16606,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -16296,6 +16654,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -16343,6 +16702,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -16390,6 +16750,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -16437,6 +16798,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -16484,6 +16846,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -16531,6 +16894,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -16578,6 +16942,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -16625,6 +16990,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -16672,6 +17038,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -16719,6 +17086,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -16766,6 +17134,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -16813,6 +17182,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -16860,6 +17230,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -16905,6 +17276,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -16952,6 +17324,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -16999,6 +17372,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -17046,6 +17420,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -17093,6 +17468,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -17140,6 +17516,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -17187,6 +17564,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -17234,6 +17612,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -17281,6 +17660,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -17326,6 +17706,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -17373,6 +17754,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -17420,6 +17802,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -17467,6 +17850,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -17514,6 +17898,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -17561,6 +17946,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -17608,6 +17994,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -17655,6 +18042,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -17702,6 +18090,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -17749,6 +18138,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -17796,6 +18186,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -17843,6 +18234,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -17888,6 +18280,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -17935,6 +18328,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -17982,6 +18376,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -18029,6 +18424,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -18074,6 +18470,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -18121,6 +18518,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -18168,6 +18566,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -18215,6 +18614,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N380" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -18262,6 +18662,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -18309,6 +18710,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N382" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -18354,6 +18756,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N383" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -18399,6 +18802,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N384" t="inlineStr"/>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -18446,6 +18850,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N385" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -18493,6 +18898,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N386" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -18540,6 +18946,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -18587,6 +18994,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -18634,6 +19042,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N389" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -18681,6 +19090,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N390" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -18728,6 +19138,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N391" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -18775,6 +19186,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -18822,6 +19234,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N393" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -18869,6 +19282,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N394" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -18916,6 +19330,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N395" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -18963,6 +19378,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -19010,6 +19426,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -19057,6 +19474,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N398" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -19104,6 +19522,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -19151,6 +19570,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N400" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -19198,6 +19618,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N401" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -19243,6 +19664,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N402" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -19290,6 +19712,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -19337,6 +19760,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N404" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -19384,6 +19808,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N405" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -19431,6 +19856,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N406" t="inlineStr"/>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -19478,6 +19904,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N407" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -19525,6 +19952,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N408" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -19572,6 +20000,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N409" t="inlineStr"/>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -19619,6 +20048,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N410" t="inlineStr"/>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -19666,6 +20096,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N411" t="inlineStr"/>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -19713,6 +20144,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N412" t="inlineStr"/>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -19760,6 +20192,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N413" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -19807,6 +20240,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N414" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -19854,6 +20288,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -19901,6 +20336,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N416" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -19948,6 +20384,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N417" t="inlineStr"/>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -19995,6 +20432,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N418" t="inlineStr"/>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -20042,6 +20480,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N419" t="inlineStr"/>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -20089,6 +20528,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N420" t="inlineStr"/>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -20134,6 +20574,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N421" t="inlineStr"/>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
@@ -20181,6 +20622,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N422" t="inlineStr"/>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -20228,6 +20670,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N423" t="inlineStr"/>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -20273,6 +20716,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N424" t="inlineStr"/>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -20320,6 +20764,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N425" t="inlineStr"/>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -20367,6 +20812,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N426" t="inlineStr"/>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -20414,6 +20860,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N427" t="inlineStr"/>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -20461,6 +20908,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N428" t="inlineStr"/>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -20506,6 +20954,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N429" t="inlineStr"/>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -20553,6 +21002,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N430" t="inlineStr"/>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -20600,6 +21050,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N431" t="inlineStr"/>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
@@ -20645,6 +21096,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N432" t="inlineStr"/>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -20692,6 +21144,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N433" t="inlineStr">
+        <is>
+          <t>Total_Cholesterol_mg_dL</t>
+        </is>
+      </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -20739,6 +21196,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N434" t="inlineStr"/>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -20786,6 +21244,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N435" t="inlineStr"/>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -20831,6 +21290,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N436" t="inlineStr"/>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -20878,6 +21338,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N437" t="inlineStr"/>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -20925,6 +21386,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N438" t="inlineStr"/>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
@@ -20972,6 +21434,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N439" t="inlineStr"/>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -21019,6 +21482,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N440" t="inlineStr"/>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
@@ -21064,6 +21528,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N441" t="inlineStr"/>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
@@ -21111,6 +21576,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N442" t="inlineStr"/>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -21156,6 +21622,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N443" t="inlineStr"/>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
@@ -21203,6 +21670,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N444" t="inlineStr"/>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -21250,6 +21718,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N445" t="inlineStr"/>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -21297,6 +21766,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N446" t="inlineStr"/>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
@@ -21344,6 +21814,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N447" t="inlineStr"/>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
@@ -21391,6 +21862,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N448" t="inlineStr"/>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
@@ -21438,6 +21910,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N449" t="inlineStr"/>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
@@ -21485,6 +21958,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N450" t="inlineStr"/>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
@@ -21532,6 +22006,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N451" t="inlineStr"/>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -21579,6 +22054,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N452" t="inlineStr"/>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
@@ -21626,6 +22102,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N453" t="inlineStr"/>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
@@ -21673,6 +22150,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N454" t="inlineStr"/>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -21720,6 +22198,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N455" t="inlineStr"/>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -21767,6 +22246,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N456" t="inlineStr"/>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
@@ -21814,6 +22294,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N457" t="inlineStr"/>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
@@ -21861,6 +22342,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N458" t="inlineStr"/>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
@@ -21908,6 +22390,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N459" t="inlineStr"/>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -21955,6 +22438,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N460" t="inlineStr"/>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -22002,6 +22486,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N461" t="inlineStr"/>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
@@ -22049,6 +22534,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N462" t="inlineStr"/>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
@@ -22096,6 +22582,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N463" t="inlineStr"/>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
@@ -22143,6 +22630,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N464" t="inlineStr"/>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -22190,6 +22678,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N465" t="inlineStr"/>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
@@ -22237,6 +22726,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N466" t="inlineStr"/>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
@@ -22284,6 +22774,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N467" t="inlineStr"/>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
@@ -22331,6 +22822,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N468" t="inlineStr"/>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
@@ -22378,6 +22870,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N469" t="inlineStr"/>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
@@ -22423,6 +22916,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N470" t="inlineStr"/>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
@@ -22470,6 +22964,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N471" t="inlineStr"/>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -22517,6 +23012,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N472" t="inlineStr"/>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
@@ -22564,6 +23060,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N473" t="inlineStr"/>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
@@ -22611,6 +23108,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N474" t="inlineStr"/>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
@@ -22658,6 +23156,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N475" t="inlineStr"/>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
@@ -22705,6 +23204,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N476" t="inlineStr"/>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
@@ -22752,6 +23252,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N477" t="inlineStr"/>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
@@ -22799,6 +23300,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N478" t="inlineStr"/>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
@@ -22846,6 +23348,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N479" t="inlineStr"/>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -22893,6 +23396,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N480" t="inlineStr"/>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
@@ -22940,6 +23444,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N481" t="inlineStr"/>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
@@ -22987,6 +23492,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N482" t="inlineStr"/>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
@@ -23032,6 +23538,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N483" t="inlineStr"/>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
@@ -23079,6 +23586,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N484" t="inlineStr"/>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
@@ -23126,6 +23634,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N485" t="inlineStr"/>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
@@ -23173,6 +23682,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N486" t="inlineStr"/>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
@@ -23220,6 +23730,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N487" t="inlineStr"/>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
@@ -23267,6 +23778,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N488" t="inlineStr"/>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
@@ -23314,6 +23826,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N489" t="inlineStr"/>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
@@ -23359,6 +23872,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N490" t="inlineStr"/>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
@@ -23404,6 +23918,11 @@
       <c r="M491" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="N491" t="inlineStr">
+        <is>
+          <t>Total_Cholesterol_mg_dL</t>
         </is>
       </c>
     </row>
@@ -23451,6 +23970,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N492" t="inlineStr"/>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -23496,6 +24016,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N493" t="inlineStr"/>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
@@ -23543,6 +24064,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N494" t="inlineStr"/>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -23590,6 +24112,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N495" t="inlineStr"/>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
@@ -23637,6 +24160,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N496" t="inlineStr">
+        <is>
+          <t>Total_Cholesterol_mg_dL</t>
+        </is>
+      </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
@@ -23684,6 +24212,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N497" t="inlineStr"/>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -23729,6 +24258,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N498" t="inlineStr"/>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -23776,6 +24306,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N499" t="inlineStr"/>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
@@ -23821,6 +24352,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N500" t="inlineStr"/>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
@@ -23868,6 +24400,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N501" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>